<commit_message>
ACL & Port Security Implemented
</commit_message>
<xml_diff>
--- a/My Plan.xlsx
+++ b/My Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mkuma\Work\CNDC Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71A9AD4D-1253-4684-8B5A-7ECA76F61AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9AFD1C-B1F7-40E9-B2C8-F1E8E570D9C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46B8CC19-4F7B-4025-B0A1-7C5423F41882}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{46B8CC19-4F7B-4025-B0A1-7C5423F41882}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="337">
-  <si>
-    <t>Campus Building</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="340">
   <si>
     <t>Department / Lab / Use</t>
   </si>
@@ -413,9 +410,6 @@
     <t>23.122.19.15</t>
   </si>
   <si>
-    <t>(Listed as 78 in Excel)</t>
-  </si>
-  <si>
     <t>23.122.19.16</t>
   </si>
   <si>
@@ -536,9 +530,6 @@
     <t>192.168.153.43</t>
   </si>
   <si>
-    <t>Media &amp; Research</t>
-  </si>
-  <si>
     <t>192.168.50.0</t>
   </si>
   <si>
@@ -638,9 +629,6 @@
     <t>Printer1</t>
   </si>
   <si>
-    <t xml:space="preserve">100 Campus </t>
-  </si>
-  <si>
     <t xml:space="preserve">CS Lab (58 PCs, 2 Pr, 1 Srv) </t>
   </si>
   <si>
@@ -677,9 +665,6 @@
     <t xml:space="preserve">Administration (4 PCs) </t>
   </si>
   <si>
-    <t xml:space="preserve">99 Campus </t>
-  </si>
-  <si>
     <t xml:space="preserve">Faculty (32 PCs, 6 Pr) </t>
   </si>
   <si>
@@ -701,9 +686,6 @@
     <t xml:space="preserve">Administration (2 PCs) </t>
   </si>
   <si>
-    <t xml:space="preserve">154 Campus </t>
-  </si>
-  <si>
     <t xml:space="preserve">Faculty (18 PCs, 2 Pr) </t>
   </si>
   <si>
@@ -716,9 +698,6 @@
     <t xml:space="preserve">Academic Dept (1 PC, 1 Pr) </t>
   </si>
   <si>
-    <t xml:space="preserve">79 Campus </t>
-  </si>
-  <si>
     <t xml:space="preserve">Library (8 PCs) </t>
   </si>
   <si>
@@ -737,9 +716,6 @@
     <t xml:space="preserve">EDC Dept (3 PCs, 1 Pr) </t>
   </si>
   <si>
-    <t xml:space="preserve">153 Campus </t>
-  </si>
-  <si>
     <t xml:space="preserve">Admission Dept (8 PCs, 3 Pr) </t>
   </si>
   <si>
@@ -747,9 +723,6 @@
   </si>
   <si>
     <t xml:space="preserve">Faculty (8 PCs, 3 Pr) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Villas </t>
   </si>
   <si>
     <t xml:space="preserve">Classrooms (3 PCs) </t>
@@ -1187,6 +1160,42 @@
   </si>
   <si>
     <t>Max Needed Hosts According to Guideline</t>
+  </si>
+  <si>
+    <t>Server</t>
+  </si>
+  <si>
+    <t>23.122.44.252</t>
+  </si>
+  <si>
+    <t>Port Security</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Campus Building/Vlan</t>
+  </si>
+  <si>
+    <t>100 Campus /10</t>
+  </si>
+  <si>
+    <t>99 Campus /10</t>
+  </si>
+  <si>
+    <t>153 Campus /10</t>
+  </si>
+  <si>
+    <t>Media &amp; Research/10</t>
+  </si>
+  <si>
+    <t>Villas /20</t>
+  </si>
+  <si>
+    <t>79 Campus /10</t>
+  </si>
+  <si>
+    <t>154 Campus /10</t>
   </si>
 </sst>
 </file>
@@ -1228,12 +1237,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1263,7 +1278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1285,6 +1300,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1622,11 +1638,11 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I210"/>
+  <dimension ref="A1:I212"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.28515625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="52" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="12.5703125" style="4" customWidth="1"/>
     <col min="4" max="4" width="18.28515625" style="4" customWidth="1"/>
     <col min="5" max="5" width="19.42578125" style="4" customWidth="1"/>
@@ -1639,1152 +1655,1226 @@
   <sheetData>
     <row r="1" spans="1:9" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>200</v>
+        <v>333</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C2" s="2">
         <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>20</v>
+      </c>
       <c r="B3" s="1" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C3" s="2">
         <v>41</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
+      <c r="I3" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>30</v>
+      </c>
       <c r="B4" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C4" s="2">
         <v>41</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
+      <c r="I4" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>40</v>
+      </c>
       <c r="B5" s="1" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C5" s="2">
         <v>37</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
+      <c r="I5" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>50</v>
+      </c>
       <c r="B6" s="1" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C6" s="2">
         <v>38</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
+      <c r="I6" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>60</v>
+      </c>
       <c r="B7" s="1" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C7" s="2">
         <v>35</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
+      <c r="I7" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>70</v>
+      </c>
       <c r="B8" s="1" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C8" s="2">
         <v>29</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="I8" s="1"/>
     </row>
-    <row r="9" spans="1:9" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
+    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>80</v>
+      </c>
       <c r="B9" s="1" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C9" s="2">
         <v>20</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
+    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>90</v>
+      </c>
       <c r="B10" s="1" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C10" s="2">
         <v>12</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="I10" s="1"/>
     </row>
-    <row r="11" spans="1:9" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
+    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>100</v>
+      </c>
       <c r="B11" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C11" s="2">
         <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
+      <c r="I11" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>110</v>
+      </c>
       <c r="B12" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C12" s="2">
         <v>8</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:9" ht="39" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
+    <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>120</v>
+      </c>
       <c r="B13" s="1" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C13" s="2">
         <v>4</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="I13" s="1"/>
     </row>
-    <row r="14" spans="1:9" ht="39" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14" s="2">
         <v>2</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="I14" s="1"/>
     </row>
-    <row r="15" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>213</v>
+        <v>334</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C15" s="2">
         <v>38</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>68</v>
-      </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
+    <row r="16" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>20</v>
+      </c>
       <c r="B16" s="1" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="C16" s="2">
         <v>18</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
+    <row r="17" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>30</v>
+      </c>
       <c r="B17" s="1" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C17" s="2">
         <v>16</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="H17" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
+    <row r="18" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>40</v>
+      </c>
       <c r="B18" s="1" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C18" s="2">
         <v>4</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
+    <row r="19" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>50</v>
+      </c>
       <c r="B19" s="1" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C19" s="2">
         <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
+    <row r="20" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>60</v>
+      </c>
       <c r="B20" s="1" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C20" s="2">
         <v>5</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="H20" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
+    <row r="21" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>70</v>
+      </c>
       <c r="B21" s="1" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C21" s="2">
         <v>2</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H21" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C22" s="2">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="H22" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>96</v>
-      </c>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>221</v>
+        <v>339</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C23" s="2">
         <v>20</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="H23" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
+    <row r="24" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>20</v>
+      </c>
       <c r="B24" s="1" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C24" s="2">
         <v>16</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="H24" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="H24" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
+      <c r="I24" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>30</v>
+      </c>
       <c r="B25" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C25" s="2">
         <v>8</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="H25" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
+    <row r="26" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>40</v>
+      </c>
       <c r="B26" s="1" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C26" s="2">
         <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F26" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="H26" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="I26" s="1"/>
     </row>
-    <row r="27" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
+    <row r="27" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>50</v>
+      </c>
       <c r="B27" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C27" s="2">
         <v>2</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="H27" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="H27" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28" s="2">
         <v>2</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="H28" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>120</v>
-      </c>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>226</v>
+        <v>338</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="C29" s="2">
         <v>8</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F29" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="G29" s="1" t="s">
+      <c r="H29" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>125</v>
+    <row r="30" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>20</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="C30" s="2">
         <v>9</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G30" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
+    <row r="31" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
       <c r="B31" s="1" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="C31" s="2">
         <v>9</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G31" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
+    <row r="32" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>40</v>
+      </c>
       <c r="B32" s="1" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C32" s="2">
         <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G32" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F32" s="1" t="s">
+      <c r="H32" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G32" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
+    <row r="33" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>50</v>
+      </c>
       <c r="B33" s="1" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C33" s="2">
         <v>5</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G33" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F33" s="1" t="s">
+      <c r="H33" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="G33" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>141</v>
-      </c>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
+    <row r="34" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>60</v>
+      </c>
       <c r="B34" s="1" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C34" s="2">
         <v>4</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F34" s="1" t="s">
+      <c r="H34" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="G34" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="I34" s="1"/>
     </row>
-    <row r="35" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C35" s="2">
         <v>2</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="G35" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F35" s="1" t="s">
+      <c r="H35" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="I35" s="1"/>
     </row>
-    <row r="36" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>233</v>
+        <v>335</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="C36" s="2">
         <v>11</v>
       </c>
       <c r="D36" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="G36" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="E36" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F36" s="1" t="s">
+      <c r="H36" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>153</v>
-      </c>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
+    <row r="37" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>20</v>
+      </c>
       <c r="B37" s="1" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="C37" s="2">
         <v>6</v>
       </c>
       <c r="D37" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G37" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>157</v>
-      </c>
       <c r="I37" s="1"/>
     </row>
-    <row r="38" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="1"/>
+    <row r="38" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>30</v>
+      </c>
       <c r="B38" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C38" s="2">
         <v>2</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="G38" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F38" s="1" t="s">
+      <c r="H38" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="G38" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="I38" s="1"/>
     </row>
-    <row r="39" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C39" s="2">
         <v>2</v>
       </c>
       <c r="D39" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="G39" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F39" s="1" t="s">
+      <c r="H39" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="G39" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>166</v>
+        <v>336</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="C40" s="2">
         <v>11</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H40" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>170</v>
-      </c>
       <c r="I40" s="1"/>
     </row>
-    <row r="41" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>237</v>
+        <v>337</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="C41" s="2">
         <v>3</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H41" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E41" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>174</v>
-      </c>
       <c r="I41" s="1"/>
     </row>
-    <row r="42" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1"/>
+    <row r="42" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>30</v>
+      </c>
       <c r="B42" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C42" s="2">
         <v>2</v>
       </c>
       <c r="D42" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="H42" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="I42" s="1"/>
     </row>
-    <row r="43" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C43" s="2">
         <v>2</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H43" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="E43" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F43" s="1" t="s">
+      <c r="I43" s="1"/>
+    </row>
+    <row r="44" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>181</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="I43" s="1"/>
-    </row>
-    <row r="44" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>184</v>
       </c>
       <c r="C44" s="2">
         <v>2</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>188</v>
-      </c>
       <c r="I44" s="3"/>
     </row>
-    <row r="45" spans="1:9" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>192</v>
-      </c>
       <c r="G45" s="1" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="I45" s="3"/>
     </row>
     <row r="48" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="B48" s="5" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.2">
@@ -2793,18 +2883,18 @@
         <v>100</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
     </row>
     <row r="50" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B50" s="7" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="D50" s="4">
         <v>100</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.2">
@@ -2813,24 +2903,24 @@
         <v>100</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="52" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B52" s="7" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
       <c r="D52" s="4">
         <v>100</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.2">
@@ -2839,30 +2929,30 @@
         <v>100</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
     </row>
     <row r="54" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B54" s="7" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="D54" s="4">
         <v>100</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.2">
@@ -2871,27 +2961,27 @@
         <v>100</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="56" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B56" s="7" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="D56" s="4">
         <v>100</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.2">
@@ -2899,24 +2989,24 @@
         <v>100</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="58" spans="2:7" ht="15" x14ac:dyDescent="0.25">
       <c r="B58" s="5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D58" s="4">
         <v>100</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.2">
@@ -2925,30 +3015,30 @@
         <v>100</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
     </row>
     <row r="60" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B60" s="7" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="D60" s="4">
         <v>100</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.2">
@@ -2957,27 +3047,27 @@
         <v>100</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
     </row>
     <row r="62" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B62" s="7" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
       <c r="D62" s="4">
         <v>100</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.2">
@@ -2986,24 +3076,24 @@
         <v>100</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="64" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B64" s="7" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="D64" s="4">
         <v>100</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.2">
@@ -3012,314 +3102,318 @@
         <v>100</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="66" spans="2:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B66" s="7" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="D66" s="4">
         <v>100</v>
       </c>
       <c r="E66" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="67" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B67" s="7"/>
+      <c r="D67" s="4">
+        <v>100</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D68" s="4">
+        <v>100</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="69" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B69" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D69" s="4">
+        <v>100</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B70" s="6"/>
+      <c r="D70" s="4">
+        <v>100</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B71" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D71" s="4">
+        <v>100</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="G71" s="4" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B72" s="6"/>
+      <c r="D72" s="4">
+        <v>100</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="73" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B73" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="D73" s="4">
+        <v>100</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B74" s="6"/>
+      <c r="D74" s="4">
+        <v>100</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B75" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="D75" s="4">
+        <v>100</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B76" s="6"/>
+      <c r="D76" s="4">
+        <v>100</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B77" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="D77" s="4">
+        <v>100</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D78" s="4">
+        <v>100</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F78" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B79" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D79" s="4">
+        <v>100</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="80" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B80" s="6"/>
+      <c r="D80" s="4">
+        <v>100</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="G80" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="F66" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="G66" s="4" t="s">
+    </row>
+    <row r="81" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B81" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="D81" s="4">
+        <v>100</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B82" s="6"/>
+      <c r="D82" s="4">
+        <v>100</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="83" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B83" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="D83" s="4">
+        <v>100</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="84" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B84" s="6"/>
+      <c r="D84" s="4">
+        <v>100</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="G84" s="4" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D67" s="4">
-        <v>100</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="F67" s="4" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="68" spans="2:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="B68" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="D68" s="4">
-        <v>100</v>
-      </c>
-      <c r="E68" s="4" t="s">
+    <row r="85" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B85" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="D85" s="4">
+        <v>100</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="86" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B86" s="6"/>
+      <c r="D86" s="4">
+        <v>100</v>
+      </c>
+      <c r="E86" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="F68" s="4" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B69" s="6"/>
-      <c r="D69" s="4">
-        <v>100</v>
-      </c>
-      <c r="E69" s="4" t="s">
+      <c r="F86" s="4" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="87" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B87" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="D87" s="4">
+        <v>100</v>
+      </c>
+      <c r="E87" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="F69" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="70" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B70" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="D70" s="4">
-        <v>100</v>
-      </c>
-      <c r="E70" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="F70" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="G70" s="4" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B71" s="6"/>
-      <c r="D71" s="4">
-        <v>100</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="F71" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="G71" s="4" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="72" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B72" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="D72" s="4">
-        <v>100</v>
-      </c>
-      <c r="E72" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="F72" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="G72" s="4" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B73" s="6"/>
-      <c r="D73" s="4">
-        <v>100</v>
-      </c>
-      <c r="E73" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="F73" s="4" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="74" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B74" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="D74" s="4">
-        <v>100</v>
-      </c>
-      <c r="E74" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="F74" s="4" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B75" s="6"/>
-      <c r="D75" s="4">
-        <v>100</v>
-      </c>
-      <c r="E75" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="76" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B76" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="D76" s="4">
-        <v>100</v>
-      </c>
-      <c r="E76" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="F76" s="4" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D77" s="4">
-        <v>100</v>
-      </c>
-      <c r="E77" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="F77" s="4" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="78" spans="2:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="B78" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="D78" s="4">
-        <v>100</v>
-      </c>
-      <c r="E78" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="F78" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B79" s="6"/>
-      <c r="D79" s="4">
-        <v>100</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="F79" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="G79" s="4" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="80" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B80" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="D80" s="4">
-        <v>100</v>
-      </c>
-      <c r="E80" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="F80" s="4" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B81" s="6"/>
-      <c r="D81" s="4">
-        <v>100</v>
-      </c>
-      <c r="E81" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="F81" s="4" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="82" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B82" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="D82" s="4">
-        <v>100</v>
-      </c>
-      <c r="E82" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="F82" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B83" s="6"/>
-      <c r="D83" s="4">
-        <v>100</v>
-      </c>
-      <c r="E83" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="F83" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="G83" s="4" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="84" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B84" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="D84" s="4">
-        <v>100</v>
-      </c>
-      <c r="E84" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="F84" s="4" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B85" s="6"/>
-      <c r="D85" s="4">
-        <v>100</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="86" spans="2:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="B86" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="D86" s="4">
-        <v>100</v>
-      </c>
-      <c r="E86" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="F86" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D87" s="4">
-        <v>100</v>
-      </c>
-      <c r="E87" s="4" t="s">
-        <v>266</v>
-      </c>
       <c r="F87" s="4" t="s">
-        <v>268</v>
+        <v>233</v>
       </c>
     </row>
     <row r="88" spans="2:7" x14ac:dyDescent="0.2">
@@ -3327,10 +3421,10 @@
         <v>100</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.2">
@@ -3338,10 +3432,10 @@
         <v>100</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="90" spans="2:7" x14ac:dyDescent="0.2">
@@ -3349,10 +3443,10 @@
         <v>100</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.2">
@@ -3360,10 +3454,10 @@
         <v>100</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.2">
@@ -3371,10 +3465,10 @@
         <v>100</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.2">
@@ -3382,10 +3476,10 @@
         <v>100</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>268</v>
+        <v>233</v>
       </c>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.2">
@@ -3393,10 +3487,10 @@
         <v>100</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
     </row>
     <row r="95" spans="2:7" x14ac:dyDescent="0.2">
@@ -3404,24 +3498,24 @@
         <v>100</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D96" s="4">
-        <v>100</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>249</v>
+      <c r="D96" s="9">
+        <v>100</v>
+      </c>
+      <c r="E96" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="F96" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G96" s="9" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="97" spans="4:7" x14ac:dyDescent="0.2">
@@ -3429,10 +3523,10 @@
         <v>100</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="98" spans="4:7" x14ac:dyDescent="0.2">
@@ -3440,10 +3534,10 @@
         <v>100</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="99" spans="4:7" x14ac:dyDescent="0.2">
@@ -3451,13 +3545,10 @@
         <v>100</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="G99" s="4" t="s">
-        <v>274</v>
+        <v>233</v>
       </c>
     </row>
     <row r="100" spans="4:7" x14ac:dyDescent="0.2">
@@ -3465,10 +3556,13 @@
         <v>100</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>249</v>
+        <v>234</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="101" spans="4:7" x14ac:dyDescent="0.2">
@@ -3476,10 +3570,10 @@
         <v>100</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="102" spans="4:7" x14ac:dyDescent="0.2">
@@ -3487,10 +3581,10 @@
         <v>100</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="103" spans="4:7" x14ac:dyDescent="0.2">
@@ -3498,10 +3592,10 @@
         <v>100</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="104" spans="4:7" x14ac:dyDescent="0.2">
@@ -3509,10 +3603,10 @@
         <v>100</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="105" spans="4:7" x14ac:dyDescent="0.2">
@@ -3520,10 +3614,10 @@
         <v>100</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="106" spans="4:7" x14ac:dyDescent="0.2">
@@ -3531,13 +3625,10 @@
         <v>100</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="G106" s="4" t="s">
-        <v>277</v>
+        <v>233</v>
       </c>
     </row>
     <row r="107" spans="4:7" x14ac:dyDescent="0.2">
@@ -3545,13 +3636,13 @@
         <v>100</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>278</v>
+        <v>196</v>
       </c>
       <c r="G107" s="4" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
     </row>
     <row r="108" spans="4:7" x14ac:dyDescent="0.2">
@@ -3559,21 +3650,24 @@
         <v>100</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>249</v>
+        <v>269</v>
+      </c>
+      <c r="G108" s="4" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="109" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D109" s="4">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>280</v>
+        <v>240</v>
       </c>
     </row>
     <row r="110" spans="4:7" x14ac:dyDescent="0.2">
@@ -3581,10 +3675,10 @@
         <v>99</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
     </row>
     <row r="111" spans="4:7" x14ac:dyDescent="0.2">
@@ -3592,10 +3686,10 @@
         <v>99</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
     </row>
     <row r="112" spans="4:7" x14ac:dyDescent="0.2">
@@ -3603,10 +3697,10 @@
         <v>99</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="113" spans="4:7" x14ac:dyDescent="0.2">
@@ -3614,10 +3708,10 @@
         <v>99</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="114" spans="4:7" x14ac:dyDescent="0.2">
@@ -3625,10 +3719,10 @@
         <v>99</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="115" spans="4:7" x14ac:dyDescent="0.2">
@@ -3636,10 +3730,10 @@
         <v>99</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="116" spans="4:7" x14ac:dyDescent="0.2">
@@ -3647,10 +3741,10 @@
         <v>99</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="117" spans="4:7" x14ac:dyDescent="0.2">
@@ -3658,24 +3752,24 @@
         <v>99</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G117" s="4" t="s">
-        <v>284</v>
+        <v>233</v>
       </c>
     </row>
     <row r="118" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D118" s="4">
+      <c r="D118" s="9">
         <v>99</v>
       </c>
-      <c r="E118" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="F118" s="4" t="s">
-        <v>249</v>
+      <c r="E118" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="F118" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="G118" s="9" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="119" spans="4:7" x14ac:dyDescent="0.2">
@@ -3683,10 +3777,10 @@
         <v>99</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="120" spans="4:7" x14ac:dyDescent="0.2">
@@ -3694,10 +3788,10 @@
         <v>99</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="121" spans="4:7" x14ac:dyDescent="0.2">
@@ -3705,13 +3799,10 @@
         <v>99</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G121" s="4" t="s">
-        <v>285</v>
+        <v>233</v>
       </c>
     </row>
     <row r="122" spans="4:7" x14ac:dyDescent="0.2">
@@ -3719,10 +3810,13 @@
         <v>99</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>249</v>
+        <v>274</v>
+      </c>
+      <c r="G122" s="4" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="123" spans="4:7" x14ac:dyDescent="0.2">
@@ -3730,10 +3824,10 @@
         <v>99</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="124" spans="4:7" x14ac:dyDescent="0.2">
@@ -3741,10 +3835,10 @@
         <v>99</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="125" spans="4:7" x14ac:dyDescent="0.2">
@@ -3752,13 +3846,10 @@
         <v>99</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G125" s="4" t="s">
-        <v>286</v>
+        <v>233</v>
       </c>
     </row>
     <row r="126" spans="4:7" x14ac:dyDescent="0.2">
@@ -3766,10 +3857,13 @@
         <v>99</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>249</v>
+        <v>274</v>
+      </c>
+      <c r="G126" s="4" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="127" spans="4:7" x14ac:dyDescent="0.2">
@@ -3777,10 +3871,10 @@
         <v>99</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="128" spans="4:7" x14ac:dyDescent="0.2">
@@ -3788,10 +3882,10 @@
         <v>99</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="129" spans="4:7" x14ac:dyDescent="0.2">
@@ -3799,10 +3893,10 @@
         <v>99</v>
       </c>
       <c r="E129" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>268</v>
+        <v>233</v>
       </c>
     </row>
     <row r="130" spans="4:7" x14ac:dyDescent="0.2">
@@ -3810,13 +3904,10 @@
         <v>99</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="G130" s="4" t="s">
-        <v>288</v>
+        <v>259</v>
       </c>
     </row>
     <row r="131" spans="4:7" x14ac:dyDescent="0.2">
@@ -3824,13 +3915,13 @@
         <v>99</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>278</v>
+        <v>196</v>
       </c>
       <c r="G131" s="4" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
     </row>
     <row r="132" spans="4:7" x14ac:dyDescent="0.2">
@@ -3838,10 +3929,13 @@
         <v>99</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>249</v>
+        <v>269</v>
+      </c>
+      <c r="G132" s="4" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="133" spans="4:7" x14ac:dyDescent="0.2">
@@ -3849,10 +3943,10 @@
         <v>99</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="134" spans="4:7" x14ac:dyDescent="0.2">
@@ -3860,10 +3954,10 @@
         <v>99</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="135" spans="4:7" x14ac:dyDescent="0.2">
@@ -3871,10 +3965,10 @@
         <v>99</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="136" spans="4:7" x14ac:dyDescent="0.2">
@@ -3882,13 +3976,10 @@
         <v>99</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>290</v>
+        <v>266</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>291</v>
-      </c>
-      <c r="G136" s="4" t="s">
-        <v>292</v>
+        <v>240</v>
       </c>
     </row>
     <row r="137" spans="4:7" x14ac:dyDescent="0.2">
@@ -3896,13 +3987,13 @@
         <v>99</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="G137" s="4" t="s">
-        <v>193</v>
+        <v>283</v>
       </c>
     </row>
     <row r="138" spans="4:7" x14ac:dyDescent="0.2">
@@ -3910,13 +4001,13 @@
         <v>99</v>
       </c>
       <c r="E138" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="G138" s="4" t="s">
-        <v>295</v>
+        <v>190</v>
       </c>
     </row>
     <row r="139" spans="4:7" x14ac:dyDescent="0.2">
@@ -3924,13 +4015,13 @@
         <v>99</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="G139" s="4" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
     </row>
     <row r="140" spans="4:7" x14ac:dyDescent="0.2">
@@ -3938,21 +4029,24 @@
         <v>99</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>249</v>
+        <v>287</v>
+      </c>
+      <c r="G140" s="4" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="141" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D141" s="4">
-        <v>154</v>
+        <v>99</v>
       </c>
       <c r="E141" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>298</v>
+        <v>240</v>
       </c>
     </row>
     <row r="142" spans="4:7" x14ac:dyDescent="0.2">
@@ -3960,10 +4054,10 @@
         <v>154</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
     </row>
     <row r="143" spans="4:7" x14ac:dyDescent="0.2">
@@ -3971,10 +4065,10 @@
         <v>154</v>
       </c>
       <c r="E143" s="4" t="s">
-        <v>266</v>
+        <v>281</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>267</v>
+        <v>290</v>
       </c>
     </row>
     <row r="144" spans="4:7" x14ac:dyDescent="0.2">
@@ -3982,10 +4076,10 @@
         <v>154</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="145" spans="4:7" x14ac:dyDescent="0.2">
@@ -3993,21 +4087,10 @@
         <v>154</v>
       </c>
       <c r="E145" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="146" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D146" s="4">
-        <v>154</v>
-      </c>
-      <c r="E146" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="F146" s="4" t="s">
-        <v>267</v>
+        <v>233</v>
       </c>
     </row>
     <row r="147" spans="4:7" x14ac:dyDescent="0.2">
@@ -4015,10 +4098,10 @@
         <v>154</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="F147" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="148" spans="4:7" x14ac:dyDescent="0.2">
@@ -4026,13 +4109,10 @@
         <v>154</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F148" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="G148" s="4" t="s">
-        <v>300</v>
+        <v>258</v>
       </c>
     </row>
     <row r="149" spans="4:7" x14ac:dyDescent="0.2">
@@ -4040,21 +4120,24 @@
         <v>154</v>
       </c>
       <c r="E149" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F149" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="150" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D150" s="4">
+      <c r="D150" s="9">
         <v>154</v>
       </c>
-      <c r="E150" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="F150" s="4" t="s">
-        <v>267</v>
+      <c r="E150" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="F150" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="G150" s="9" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="151" spans="4:7" x14ac:dyDescent="0.2">
@@ -4062,13 +4145,10 @@
         <v>154</v>
       </c>
       <c r="E151" s="4" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="F151" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="G151" s="4" t="s">
-        <v>301</v>
+        <v>240</v>
       </c>
     </row>
     <row r="152" spans="4:7" x14ac:dyDescent="0.2">
@@ -4076,10 +4156,10 @@
         <v>154</v>
       </c>
       <c r="E152" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F152" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
     </row>
     <row r="153" spans="4:7" x14ac:dyDescent="0.2">
@@ -4087,10 +4167,13 @@
         <v>154</v>
       </c>
       <c r="E153" s="4" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="F153" s="4" t="s">
-        <v>267</v>
+        <v>196</v>
+      </c>
+      <c r="G153" s="4" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="154" spans="4:7" x14ac:dyDescent="0.2">
@@ -4098,10 +4181,10 @@
         <v>154</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="F154" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="155" spans="4:7" x14ac:dyDescent="0.2">
@@ -4109,10 +4192,10 @@
         <v>154</v>
       </c>
       <c r="E155" s="4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="F155" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
     </row>
     <row r="156" spans="4:7" x14ac:dyDescent="0.2">
@@ -4120,10 +4203,10 @@
         <v>154</v>
       </c>
       <c r="E156" s="4" t="s">
-        <v>302</v>
+        <v>266</v>
       </c>
       <c r="F156" s="4" t="s">
-        <v>267</v>
+        <v>233</v>
       </c>
     </row>
     <row r="157" spans="4:7" x14ac:dyDescent="0.2">
@@ -4131,10 +4214,10 @@
         <v>154</v>
       </c>
       <c r="E157" s="4" t="s">
-        <v>302</v>
+        <v>266</v>
       </c>
       <c r="F157" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="158" spans="4:7" x14ac:dyDescent="0.2">
@@ -4142,13 +4225,10 @@
         <v>154</v>
       </c>
       <c r="E158" s="4" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="F158" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="G158" s="4" t="s">
-        <v>304</v>
+        <v>258</v>
       </c>
     </row>
     <row r="159" spans="4:7" x14ac:dyDescent="0.2">
@@ -4156,32 +4236,35 @@
         <v>154</v>
       </c>
       <c r="E159" s="4" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="F159" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="160" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D160" s="4">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E160" s="4" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="F160" s="4" t="s">
-        <v>305</v>
+        <v>294</v>
+      </c>
+      <c r="G160" s="4" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="161" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D161" s="4">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E161" s="4" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="F161" s="4" t="s">
-        <v>306</v>
+        <v>240</v>
       </c>
     </row>
     <row r="162" spans="4:7" x14ac:dyDescent="0.2">
@@ -4189,10 +4272,10 @@
         <v>153</v>
       </c>
       <c r="E162" s="4" t="s">
-        <v>266</v>
+        <v>293</v>
       </c>
       <c r="F162" s="4" t="s">
-        <v>267</v>
+        <v>296</v>
       </c>
     </row>
     <row r="163" spans="4:7" x14ac:dyDescent="0.2">
@@ -4200,10 +4283,10 @@
         <v>153</v>
       </c>
       <c r="E163" s="4" t="s">
-        <v>266</v>
+        <v>293</v>
       </c>
       <c r="F163" s="4" t="s">
-        <v>242</v>
+        <v>297</v>
       </c>
     </row>
     <row r="164" spans="4:7" x14ac:dyDescent="0.2">
@@ -4211,10 +4294,10 @@
         <v>153</v>
       </c>
       <c r="E164" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="F164" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
     </row>
     <row r="165" spans="4:7" x14ac:dyDescent="0.2">
@@ -4222,10 +4305,10 @@
         <v>153</v>
       </c>
       <c r="E165" s="4" t="s">
-        <v>307</v>
+        <v>257</v>
       </c>
       <c r="F165" s="4" t="s">
-        <v>267</v>
+        <v>233</v>
       </c>
     </row>
     <row r="166" spans="4:7" x14ac:dyDescent="0.2">
@@ -4233,10 +4316,10 @@
         <v>153</v>
       </c>
       <c r="E166" s="4" t="s">
-        <v>307</v>
+        <v>257</v>
       </c>
       <c r="F166" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="167" spans="4:7" x14ac:dyDescent="0.2">
@@ -4244,13 +4327,10 @@
         <v>153</v>
       </c>
       <c r="E167" s="4" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="F167" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G167" s="4" t="s">
-        <v>308</v>
+        <v>258</v>
       </c>
     </row>
     <row r="168" spans="4:7" x14ac:dyDescent="0.2">
@@ -4258,10 +4338,10 @@
         <v>153</v>
       </c>
       <c r="E168" s="4" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="F168" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="169" spans="4:7" x14ac:dyDescent="0.2">
@@ -4269,10 +4349,13 @@
         <v>153</v>
       </c>
       <c r="E169" s="4" t="s">
-        <v>273</v>
+        <v>298</v>
       </c>
       <c r="F169" s="4" t="s">
-        <v>267</v>
+        <v>274</v>
+      </c>
+      <c r="G169" s="4" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="170" spans="4:7" x14ac:dyDescent="0.2">
@@ -4280,13 +4363,10 @@
         <v>153</v>
       </c>
       <c r="E170" s="4" t="s">
-        <v>273</v>
+        <v>298</v>
       </c>
       <c r="F170" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G170" s="4" t="s">
-        <v>309</v>
+        <v>240</v>
       </c>
     </row>
     <row r="171" spans="4:7" x14ac:dyDescent="0.2">
@@ -4294,32 +4374,35 @@
         <v>153</v>
       </c>
       <c r="E171" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F171" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
     </row>
     <row r="172" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D172" s="4">
-        <v>78</v>
+        <v>153</v>
       </c>
       <c r="E172" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F172" s="4" t="s">
-        <v>310</v>
+        <v>274</v>
+      </c>
+      <c r="G172" s="4" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="173" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D173" s="4">
-        <v>78</v>
+        <v>153</v>
       </c>
       <c r="E173" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F173" s="4" t="s">
-        <v>311</v>
+        <v>240</v>
       </c>
     </row>
     <row r="174" spans="4:7" x14ac:dyDescent="0.2">
@@ -4327,10 +4410,10 @@
         <v>78</v>
       </c>
       <c r="E174" s="4" t="s">
-        <v>312</v>
+        <v>264</v>
       </c>
       <c r="F174" s="4" t="s">
-        <v>267</v>
+        <v>301</v>
       </c>
     </row>
     <row r="175" spans="4:7" x14ac:dyDescent="0.2">
@@ -4338,10 +4421,10 @@
         <v>78</v>
       </c>
       <c r="E175" s="4" t="s">
-        <v>312</v>
+        <v>264</v>
       </c>
       <c r="F175" s="4" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
     </row>
     <row r="176" spans="4:7" x14ac:dyDescent="0.2">
@@ -4349,10 +4432,10 @@
         <v>78</v>
       </c>
       <c r="E176" s="4" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
     </row>
     <row r="177" spans="4:7" x14ac:dyDescent="0.2">
@@ -4360,10 +4443,10 @@
         <v>78</v>
       </c>
       <c r="E177" s="4" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="F177" s="4" t="s">
-        <v>267</v>
+        <v>233</v>
       </c>
     </row>
     <row r="178" spans="4:7" x14ac:dyDescent="0.2">
@@ -4371,10 +4454,10 @@
         <v>78</v>
       </c>
       <c r="E178" s="4" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="F178" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="179" spans="4:7" x14ac:dyDescent="0.2">
@@ -4382,13 +4465,10 @@
         <v>78</v>
       </c>
       <c r="E179" s="4" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="F179" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G179" s="4" t="s">
-        <v>314</v>
+        <v>258</v>
       </c>
     </row>
     <row r="180" spans="4:7" x14ac:dyDescent="0.2">
@@ -4396,10 +4476,10 @@
         <v>78</v>
       </c>
       <c r="E180" s="4" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="F180" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="181" spans="4:7" x14ac:dyDescent="0.2">
@@ -4407,10 +4487,13 @@
         <v>78</v>
       </c>
       <c r="E181" s="4" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="F181" s="4" t="s">
-        <v>267</v>
+        <v>274</v>
+      </c>
+      <c r="G181" s="4" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="182" spans="4:7" x14ac:dyDescent="0.2">
@@ -4418,10 +4501,10 @@
         <v>78</v>
       </c>
       <c r="E182" s="4" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="F182" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="183" spans="4:7" x14ac:dyDescent="0.2">
@@ -4429,13 +4512,10 @@
         <v>78</v>
       </c>
       <c r="E183" s="4" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="F183" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G183" s="4" t="s">
-        <v>316</v>
+        <v>258</v>
       </c>
     </row>
     <row r="184" spans="4:7" x14ac:dyDescent="0.2">
@@ -4443,10 +4523,10 @@
         <v>78</v>
       </c>
       <c r="E184" s="4" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="F184" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="185" spans="4:7" x14ac:dyDescent="0.2">
@@ -4454,10 +4534,13 @@
         <v>78</v>
       </c>
       <c r="E185" s="4" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="F185" s="4" t="s">
-        <v>267</v>
+        <v>274</v>
+      </c>
+      <c r="G185" s="4" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="186" spans="4:7" x14ac:dyDescent="0.2">
@@ -4465,10 +4548,10 @@
         <v>78</v>
       </c>
       <c r="E186" s="4" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="F186" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="187" spans="4:7" x14ac:dyDescent="0.2">
@@ -4476,13 +4559,10 @@
         <v>78</v>
       </c>
       <c r="E187" s="4" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="F187" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G187" s="4" t="s">
-        <v>318</v>
+        <v>258</v>
       </c>
     </row>
     <row r="188" spans="4:7" x14ac:dyDescent="0.2">
@@ -4490,10 +4570,10 @@
         <v>78</v>
       </c>
       <c r="E188" s="4" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="F188" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="189" spans="4:7" x14ac:dyDescent="0.2">
@@ -4501,10 +4581,13 @@
         <v>78</v>
       </c>
       <c r="E189" s="4" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="F189" s="4" t="s">
-        <v>267</v>
+        <v>274</v>
+      </c>
+      <c r="G189" s="4" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="190" spans="4:7" x14ac:dyDescent="0.2">
@@ -4512,10 +4595,10 @@
         <v>78</v>
       </c>
       <c r="E190" s="4" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="F190" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="191" spans="4:7" x14ac:dyDescent="0.2">
@@ -4523,13 +4606,10 @@
         <v>78</v>
       </c>
       <c r="E191" s="4" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G191" s="4" t="s">
-        <v>320</v>
+        <v>258</v>
       </c>
     </row>
     <row r="192" spans="4:7" x14ac:dyDescent="0.2">
@@ -4537,10 +4617,10 @@
         <v>78</v>
       </c>
       <c r="E192" s="4" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="F192" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="193" spans="4:7" x14ac:dyDescent="0.2">
@@ -4548,10 +4628,13 @@
         <v>78</v>
       </c>
       <c r="E193" s="4" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="F193" s="4" t="s">
-        <v>267</v>
+        <v>274</v>
+      </c>
+      <c r="G193" s="4" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="194" spans="4:7" x14ac:dyDescent="0.2">
@@ -4559,10 +4642,10 @@
         <v>78</v>
       </c>
       <c r="E194" s="4" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="F194" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="195" spans="4:7" x14ac:dyDescent="0.2">
@@ -4570,13 +4653,10 @@
         <v>78</v>
       </c>
       <c r="E195" s="4" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="F195" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G195" s="4" t="s">
-        <v>322</v>
+        <v>258</v>
       </c>
     </row>
     <row r="196" spans="4:7" x14ac:dyDescent="0.2">
@@ -4584,170 +4664,195 @@
         <v>78</v>
       </c>
       <c r="E196" s="4" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="F196" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="197" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D197" s="4" t="s">
-        <v>323</v>
+      <c r="D197" s="4">
+        <v>78</v>
       </c>
       <c r="E197" s="4" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="F197" s="4" t="s">
-        <v>324</v>
+        <v>274</v>
+      </c>
+      <c r="G197" s="4" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="198" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D198" s="4" t="s">
-        <v>323</v>
+      <c r="D198" s="4">
+        <v>78</v>
       </c>
       <c r="E198" s="4" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="F198" s="4" t="s">
-        <v>325</v>
+        <v>240</v>
       </c>
     </row>
     <row r="199" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D199" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E199" s="4" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="F199" s="4" t="s">
-        <v>267</v>
+        <v>315</v>
       </c>
     </row>
     <row r="200" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D200" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E200" s="4" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="F200" s="4" t="s">
-        <v>242</v>
+        <v>316</v>
       </c>
     </row>
     <row r="201" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D201" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E201" s="4" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="F201" s="4" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
     </row>
     <row r="202" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D202" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E202" s="4" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="F202" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
     </row>
     <row r="203" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D203" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E203" s="4" t="s">
-        <v>271</v>
+        <v>317</v>
       </c>
       <c r="F203" s="4" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="204" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D204" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E204" s="4" t="s">
-        <v>271</v>
+        <v>317</v>
       </c>
       <c r="F204" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="205" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D205" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E205" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F205" s="4" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
     </row>
     <row r="206" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D206" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E206" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F206" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G206" s="4" t="s">
-        <v>327</v>
+        <v>233</v>
       </c>
     </row>
     <row r="207" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D207" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E207" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F207" s="4" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
     </row>
     <row r="208" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D208" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="E208" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="F208" s="4" t="s">
-        <v>267</v>
+      <c r="D208" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="E208" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="F208" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="G208" s="9" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="209" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D209" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E209" s="4" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="F209" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="G209" s="4" t="s">
-        <v>328</v>
+        <v>240</v>
       </c>
     </row>
     <row r="210" spans="4:7" x14ac:dyDescent="0.2">
       <c r="D210" s="4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E210" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F210" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
+      </c>
+    </row>
+    <row r="211" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="D211" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="E211" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F211" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="G211" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="212" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="D212" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="E212" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F212" s="4" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>